<commit_message>
docs(optum-rwd): refresh row 17 (payer_category) — NPPES now in scope
Vendor has confirmed Optum extract preserves dispenser/prescriber/rendering/
facility NPIs, so the prior "specialty pharmacy not directly in Optum"
pessimism is stale. Row 17 now references:
- #154 (PR B-prime: NPPES NPI taxonomy enrichment) — owns the specialty_pharmacy
  flag derivation via NUCC taxonomy codes 3336S0011X / 3336M0002X / 3336H0001X
- #156 (PR B) item 6 — owns the bus/product/health_exch/lis_dual payer_category
  derivation and column migration

Also notes the broader benefit of NPPES integration (unlocks ~8 currently-None
hcp_profiles fields, sharpens §7.7 provider-mix features) so it's not framed
as a one-off pharmacy lookup.

https://claude.ai/code/session_01DnaGVUfGXbcC55W8MqeaKL
</commit_message>
<xml_diff>
--- a/docs/data/gap_analysis/Questions_around_Gap_features_annotated.xlsx
+++ b/docs/data/gap_analysis/Questions_around_Gap_features_annotated.xlsx
@@ -1303,11 +1303,15 @@
 - scripts/rwd_common.py:43-47 has only the basic 3-way INSURANCE_TYPE_MAP (COM/MCR/MCD). This needs extension to capture lis_dual + health_exch.
 - convert_optum_rwd.py:801 calls rwdc.insurance_type(demo_row.get('bus')) -- single field; does not consume lis_dual or health_exch yet.
 - patient_journeys.insurance_type is VARCHAR(20) and does not yet have a payer_category companion column. Schema migration required (or repurpose insurance_type with widened vocabulary).
-SPECIALTY PHARMACY CHANNEL — NOT DIRECTLY IN OPTUM:
-Closest signals are:
-(a) Pharmacy NPI taxonomy code 333600000X — but Optum medication.parquet does not reliably carry the dispenser NPI in our extracts.
-(b) NDC + place-of-service combo — but place_of_service is sparsely populated.
-WORKAROUND: If your Optum extract includes dispenser_npi or pharm_npi, cross-reference against NPPES (CMS NPI registry, free monthly download). Without that, leave specialty_pharmacy_flag NULL.
+- TRACKED: GitHub issue #156 (PR B) item 6 covers the bus/product/health_exch/lis_dual derivation and the payer_category column migration.
+SPECIALTY PHARMACY CHANNEL — TRACTABLE VIA NPPES (vendor has confirmed NPI preservation in our extract):
+The earlier assumption that Optum drops the dispenser NPI was wrong — vendor confirmed dispenser/prescriber/rendering/facility NPIs are all preserved. NPPES (CMS National Plan and Provider Enumeration System) is a free public API + monthly bulk dump that gives us NUCC taxonomy codes per NPI.
+APPROACH:
+(a) Ingest the monthly NPPES bulk dump (~10 GB) into a local npi_taxonomy table; refresh monthly via Celery beat.
+(b) Resolve each medication.dispenser_npi against the cache; match NUCC taxonomy codes 3336S0011X (Specialty Pharmacy), 3336M0002X (Mail Order Pharmacy — frequently specialty), 3336H0001X (Home Infusion Therapy Pharmacy — frequently specialty). Set specialty_pharmacy_flag = TRUE on any match.
+(c) API fallback for cache-miss NPIs: https://npiregistry.cms.hhs.gov/api/?number=&lt;NPI&gt;&amp;version=2.1 (free, no auth, rate-limited — fine for new-NPI deltas).
+TRACKED: GitHub issue #154 (PR B-prime: NPPES NPI taxonomy enrichment) carries the full scope — specialty_pharmacy_flag derivation lands as item 5 of that PR.
+BONUS: the same NPPES integration unlocks ~8 currently-None fields on hcp_profiles (specialty, sub_specialty, practice_type, practice_size, years_experience, affiliation_primary, state/city/zip_code, geographic_region, academic_hcp) and sharpens §7.7 provider-mix features. Foundational ETL capability, not a one-off pharmacy flag lookup.
 BEST PRACTICE — STORE GRANULAR + NORMALIZED:
 Persist BOTH the raw source fields (bus, product, health_exch, lis_dual) AS-IS on patient_journeys AND the derived normalized payer_category. This enables future re-derivation without re-ETL and preserves audit trail. Reference the v3 schema's source_combination_method column (e2i_v3:858) as the existing precedent for keeping raw + derived together.</t>
         </is>

</xml_diff>